<commit_message>
Chat CH-2: add isolated connector and tenant capture
</commit_message>
<xml_diff>
--- a/docs_v2/OS_PLUS_V2_QA_Test_Matrix.xlsx
+++ b/docs_v2/OS_PLUS_V2_QA_Test_Matrix.xlsx
@@ -3406,7 +3406,7 @@
         <x:v>Evidence / Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="190" customHeight="1">
       <x:c r="A2" s="17" t="str">
         <x:v>BA-001</x:v>
       </x:c>
@@ -3446,11 +3446,14 @@
       <x:c r="M2" s="17" t="str">
         <x:v>Authenticated Owner/Admin opened Phantom Threads dashboard.</x:v>
       </x:c>
-      <x:c r="N2" s="17" t="str">
-        <x:v>Browser: localhost:3000/dashboard; Tenant Phantom Threads; role Owner/Admin.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
+      <x:c r="N2" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Browser: localhost:3000/dashboard; Tenant Phantom Threads; role Owner/Admin.
+CH-2 2026-10-21: Owner-a existing authenticated session and tenant selector -&gt; Local QA A verified; fresh Clerk credential entry not repeated. See docs_chat/CH2_BOUTIQUE_QA.md BA-001. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="190" customHeight="1">
       <x:c r="A3" s="17" t="str">
         <x:v>BA-002</x:v>
       </x:c>
@@ -3490,11 +3493,14 @@
       <x:c r="M3" s="17" t="str">
         <x:v>Created V2 QA Customer 20260705 and found it via phone suggestion.</x:v>
       </x:c>
-      <x:c r="N3" s="17" t="str">
-        <x:v>Customer ID bce5cbcb-c562-46c3-b960-e3204ab61a0f; phone search 9000000705 returned customer.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
+      <x:c r="N3" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Customer ID bce5cbcb-c562-46c3-b960-e3204ab61a0f; phone search 9000000705 returned customer.
+CH-2 2026-10-21: Owner scenario: created CH2 Regression Customer and exact name search returned one match. Independent Manager session not tested. See docs_chat/CH2_BOUTIQUE_QA.md BA-002. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="190" customHeight="1">
       <x:c r="A4" s="17" t="str">
         <x:v>BA-003</x:v>
       </x:c>
@@ -3534,11 +3540,14 @@
       <x:c r="M4" s="17" t="str">
         <x:v>Created default Shirt measurement and verified order-form fit reference.</x:v>
       </x:c>
-      <x:c r="N4" s="17" t="str">
-        <x:v>Measurement ID 5c2462b5-ad77-4c7b-9d81-b79db903b0d9; Chest 40, Length 28; default=true.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
+      <x:c r="N4" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Measurement ID 5c2462b5-ad77-4c7b-9d81-b79db903b0d9; Chest 40, Length 28; default=true.
+CH-2 2026-10-21: Owner scenario: saved and selected garment measurement Chest 37 for both items. Dialog stays open after save, persistence passes. See docs_chat/CH2_BOUTIQUE_QA.md BA-003. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="190" customHeight="1">
       <x:c r="A5" s="17" t="str">
         <x:v>BA-004</x:v>
       </x:c>
@@ -3578,11 +3587,14 @@
       <x:c r="M5" s="17" t="str">
         <x:v>Created Boutique order with one item using legacy order_items runtime.</x:v>
       </x:c>
-      <x:c r="N5" s="17" t="str">
-        <x:v>ORD-000011 / order 2d61e296-5cbd-4ca1-9d80-40c4da6bb7aa; item 52fb87ae-3604-48c4-8480-ac76dafb25b8.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
+      <x:c r="N5" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ORD-000011 / order 2d61e296-5cbd-4ca1-9d80-40c4da6bb7aa; item 52fb87ae-3604-48c4-8480-ac76dafb25b8.
+CH-2 2026-10-21: Owner scenario: created ORD-000002 / CHAT-CH2-BROWSER-QA, total 2000. See docs_chat/CH2_BOUTIQUE_QA.md BA-004. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="190" customHeight="1">
       <x:c r="A6" s="17" t="str">
         <x:v>BA-005</x:v>
       </x:c>
@@ -3622,11 +3634,14 @@
       <x:c r="M6" s="17" t="str">
         <x:v>Created two-item Boutique order with different workflows.</x:v>
       </x:c>
-      <x:c r="N6" s="17" t="str">
-        <x:v>ORD-000012 / order 3b27cca4-6796-46cb-b157-0890d109a4ee; two order_items with Default and Painting 1 workflow IDs.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
+      <x:c r="N6" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ORD-000012 / order 3b27cca4-6796-46cb-b157-0890d109a4ee; two order_items with Default and Painting 1 workflow IDs.
+CH-2 2026-10-21: Owner scenario: two items 1200 + 800, each with a different workflow. See docs_chat/CH2_BOUTIQUE_QA.md BA-005. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="190" customHeight="1">
       <x:c r="A7" s="17" t="str">
         <x:v>BA-006</x:v>
       </x:c>
@@ -3666,11 +3681,14 @@
       <x:c r="M7" s="17" t="str">
         <x:v>Verified workflow instances exist for created order items.</x:v>
       </x:c>
-      <x:c r="N7" s="17" t="str">
-        <x:v>ORD-000011 and ORD-000012 item_workflow_instances present via Supabase read-only check.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
+      <x:c r="N7" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ORD-000011 and ORD-000012 item_workflow_instances present via Supabase read-only check.
+CH-2 2026-10-21: Two independent workflow instances / four stage rows verified after actual UI create. See docs_chat/CH2_BOUTIQUE_QA.md BA-006. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="190" customHeight="1">
       <x:c r="A8" s="17" t="str">
         <x:v>BA-007</x:v>
       </x:c>
@@ -3710,11 +3728,14 @@
       <x:c r="M8" s="17" t="str">
         <x:v>Started Design stage with allowed Designer worker.</x:v>
       </x:c>
-      <x:c r="N8" s="17" t="str">
-        <x:v>Workflow page showed only allowed worker Designer for Design; history recorded stage started.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
+      <x:c r="N8" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Workflow page showed only allowed worker Designer for Design; history recorded stage started.
+CH-2 2026-10-21: Owner scenario: started QA prepare using Synthetic QA worker and QA workgroup. See docs_chat/CH2_BOUTIQUE_QA.md BA-007. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="190" customHeight="1">
       <x:c r="A9" s="17" t="str">
         <x:v>BA-008</x:v>
       </x:c>
@@ -3754,11 +3775,14 @@
       <x:c r="M9" s="17" t="str">
         <x:v>Completed Design stage and Cutting became ready.</x:v>
       </x:c>
-      <x:c r="N9" s="17" t="str">
-        <x:v>Workflow page showed item in production, 1/5 stages complete, Cutting ready_to_start.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
+      <x:c r="N9" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Workflow page showed item in production, 1/5 stages complete, Cutting ready_to_start.
+CH-2 2026-10-21: Completed first stage in UI; next stage ready; other item unchanged. See docs_chat/CH2_BOUTIQUE_QA.md BA-008. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="190" customHeight="1">
       <x:c r="A10" s="17" t="str">
         <x:v>BA-009</x:v>
       </x:c>
@@ -3798,11 +3822,14 @@
       <x:c r="M10" s="17" t="str">
         <x:v>Opened public tracking link and verified customer-safe status.</x:v>
       </x:c>
-      <x:c r="N10" s="17" t="str">
-        <x:v>Tracking /track/TILaKurOoqN2o_dzXhSKK-cbmZkTos5D showed ORD-000011 and item status without internal worker data.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
+      <x:c r="N10" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tracking /track/TILaKurOoqN2o_dzXhSKK-cbmZkTos5D showed ORD-000011 and item status without internal worker data.
+CH-2 2026-10-21: Public tracking page rendered safe order/item status without internal worker, stage, payment or notes. Browser retained login; no fresh anonymous browser claim. See docs_chat/CH2_BOUTIQUE_QA.md BA-009. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="190" customHeight="1">
       <x:c r="A11" s="17" t="str">
         <x:v>BA-010</x:v>
       </x:c>
@@ -3842,11 +3869,14 @@
       <x:c r="M11" s="17" t="str">
         <x:v>Recorded partial payment during order creation and verified order_payments/payment status.</x:v>
       </x:c>
-      <x:c r="N11" s="17" t="str">
-        <x:v>ORD-000011 amount_paid 200, partially_paid; ORD-000012 amount_paid 300, partially_paid.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
+      <x:c r="N11" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ORD-000011 amount_paid 200, partially_paid; ORD-000012 amount_paid 300, partially_paid.
+CH-2 2026-10-21: Owner scenario: one synthetic partial receipt 300, balance 1700; no money moved. See docs_chat/CH2_BOUTIQUE_QA.md BA-010. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="190" customHeight="1">
       <x:c r="A12" s="17" t="str">
         <x:v>BA-011</x:v>
       </x:c>
@@ -3886,11 +3916,14 @@
       <x:c r="M12" s="17" t="str">
         <x:v>Finance reflected order payment in cash/receivable totals.</x:v>
       </x:c>
-      <x:c r="N12" s="17" t="str">
-        <x:v>Finance GST page showed Cash in 200 for MTD and ORD-000011 receivable/payment summary.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
+      <x:c r="N12" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Finance GST page showed Cash in 200 for MTD and ORD-000011 receivable/payment summary.
+CH-2 2026-10-21: Owner scenario: Finance showed order collection 300 and receivable 1700. Independent Finance-role session not tested. See docs_chat/CH2_BOUTIQUE_QA.md BA-011. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="190" customHeight="1">
       <x:c r="A13" s="17" t="str">
         <x:v>BA-012</x:v>
       </x:c>
@@ -3930,11 +3963,14 @@
       <x:c r="M13" s="17" t="str">
         <x:v>GST report loaded and included GST-bearing QA order.</x:v>
       </x:c>
-      <x:c r="N13" s="17" t="str">
-        <x:v>Finance GST page showed Output GST 180 and ORD-000011 in output GST list; XLSX export link present.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
+      <x:c r="N13" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Finance GST page showed Output GST 180 and ORD-000011 in output GST list; XLSX export link present.
+CH-2 2026-10-21: Owner scenario: GST report loaded and included non-GST order when selected. Zero-GST local fixture only: GST-bearing calculation, export and filing NOT tested. See docs_chat/CH2_BOUTIQUE_QA.md BA-012. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="190" customHeight="1">
       <x:c r="A14" s="17" t="str">
         <x:v>BA-013</x:v>
       </x:c>
@@ -3974,11 +4010,14 @@
       <x:c r="M14" s="17" t="str">
         <x:v>Queued sandbox WhatsApp tracking-link message and audit log.</x:v>
       </x:c>
-      <x:c r="N14" s="17" t="str">
-        <x:v>communication_message_queue a2b4882e-e3b6-4616-bc2b-a57acc4ae030; log 8ebc4c2f-d2f2-48a5-8454-3620b8d43cdd; no live send.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
+      <x:c r="N14" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">communication_message_queue a2b4882e-e3b6-4616-bc2b-a57acc4ae030; log 8ebc4c2f-d2f2-48a5-8454-3620b8d43cdd; no live send.
+CH-2 2026-10-21: Owner scenario: UI queued email tracking dry-run to ch2-qa@example.invalid; database dryRun=true and audit verified. No message delivered. See docs_chat/CH2_BOUTIQUE_QA.md BA-013. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="190" customHeight="1">
       <x:c r="A15" s="17" t="str">
         <x:v>BA-014</x:v>
       </x:c>
@@ -4018,8 +4057,11 @@
       <x:c r="M15" s="17" t="str">
         <x:v>Opened order detail/edit shell and saved harmless order notes edit.</x:v>
       </x:c>
-      <x:c r="N15" s="17" t="str">
-        <x:v>ORD-000012 notes updated to include "Edit smoke passed" without recalculating finance/production history.</x:v>
+      <x:c r="N15" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ORD-000012 notes updated to include "Edit smoke passed" without recalculating finance/production history.
+CH-2 2026-10-21: Owner scenario: edited order notes and reopened detail, total/payment/workflow preserved. See docs_chat/CH2_BOUTIQUE_QA.md BA-014. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+        </x:is>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Chat CH-3: add tenant contacts leads and atomic customer commands
</commit_message>
<xml_diff>
--- a/docs_v2/OS_PLUS_V2_QA_Test_Matrix.xlsx
+++ b/docs_v2/OS_PLUS_V2_QA_Test_Matrix.xlsx
@@ -3406,7 +3406,7 @@
         <x:v>Evidence / Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="190" customHeight="1">
+    <x:row r="2" ht="260" customHeight="1">
       <x:c r="A2" s="17" t="str">
         <x:v>BA-001</x:v>
       </x:c>
@@ -3449,11 +3449,12 @@
       <x:c r="N2" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Browser: localhost:3000/dashboard; Tenant Phantom Threads; role Owner/Admin.
-CH-2 2026-10-21: Owner-a existing authenticated session and tenant selector -&gt; Local QA A verified; fresh Clerk credential entry not repeated. See docs_chat/CH2_BOUTIQUE_QA.md BA-001. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+CH-2 2026-10-21: Owner-a existing authenticated session and tenant selector -&gt; Local QA A verified; fresh Clerk credential entry not repeated. See docs_chat/CH2_BOUTIQUE_QA.md BA-001. Historical V2-0 status/persona preconditions are not recertified.
+CH-3 2026-10-21 owner scenario: Existing owner-a Clerk session; switched A to B and back. B cannot open new A order (404). See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="3" ht="190" customHeight="1">
+    <x:row r="3" ht="260" customHeight="1">
       <x:c r="A3" s="17" t="str">
         <x:v>BA-002</x:v>
       </x:c>
@@ -3496,11 +3497,12 @@
       <x:c r="N3" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Customer ID bce5cbcb-c562-46c3-b960-e3204ab61a0f; phone search 9000000705 returned customer.
-CH-2 2026-10-21: Owner scenario: created CH2 Regression Customer and exact name search returned one match. Independent Manager session not tested. See docs_chat/CH2_BOUTIQUE_QA.md BA-002. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+CH-2 2026-10-21: Owner scenario: created CH2 Regression Customer and exact name search returned one match. Independent Manager session not tested. See docs_chat/CH2_BOUTIQUE_QA.md BA-002. Historical V2-0 status/persona preconditions are not recertified.
+CH-3 2026-10-21 owner scenario: Created CH3 Regression Customer; exact-name search returns one result. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="4" ht="190" customHeight="1">
+    <x:row r="4" ht="260" customHeight="1">
       <x:c r="A4" s="17" t="str">
         <x:v>BA-003</x:v>
       </x:c>
@@ -3543,11 +3545,12 @@
       <x:c r="N4" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Measurement ID 5c2462b5-ad77-4c7b-9d81-b79db903b0d9; Chest 40, Length 28; default=true.
-CH-2 2026-10-21: Owner scenario: saved and selected garment measurement Chest 37 for both items. Dialog stays open after save, persistence passes. See docs_chat/CH2_BOUTIQUE_QA.md BA-003. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+CH-2 2026-10-21: Owner scenario: saved and selected garment measurement Chest 37 for both items. Dialog stays open after save, persistence passes. See docs_chat/CH2_BOUTIQUE_QA.md BA-003. Historical V2-0 status/persona preconditions are not recertified.
+CH-3 2026-10-21 owner scenario: Saved default CH3 garment fit Chest38; selected on both items. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="5" ht="190" customHeight="1">
+    <x:row r="5" ht="260" customHeight="1">
       <x:c r="A5" s="17" t="str">
         <x:v>BA-004</x:v>
       </x:c>
@@ -3590,11 +3593,12 @@
       <x:c r="N5" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">ORD-000011 / order 2d61e296-5cbd-4ca1-9d80-40c4da6bb7aa; item 52fb87ae-3604-48c4-8480-ac76dafb25b8.
-CH-2 2026-10-21: Owner scenario: created ORD-000002 / CHAT-CH2-BROWSER-QA, total 2000. See docs_chat/CH2_BOUTIQUE_QA.md BA-004. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+CH-2 2026-10-21: Owner scenario: created ORD-000002 / CHAT-CH2-BROWSER-QA, total 2000. See docs_chat/CH2_BOUTIQUE_QA.md BA-004. Historical V2-0 status/persona preconditions are not recertified.
+CH-3 2026-10-21 owner scenario: Created ORD-000003 / CHAT-CH3-BROWSER-QA total2000. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="6" ht="190" customHeight="1">
+    <x:row r="6" ht="260" customHeight="1">
       <x:c r="A6" s="17" t="str">
         <x:v>BA-005</x:v>
       </x:c>
@@ -3637,11 +3641,12 @@
       <x:c r="N6" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">ORD-000012 / order 3b27cca4-6796-46cb-b157-0890d109a4ee; two order_items with Default and Painting 1 workflow IDs.
-CH-2 2026-10-21: Owner scenario: two items 1200 + 800, each with a different workflow. See docs_chat/CH2_BOUTIQUE_QA.md BA-005. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+CH-2 2026-10-21: Owner scenario: two items 1200 + 800, each with a different workflow. See docs_chat/CH2_BOUTIQUE_QA.md BA-005. Historical V2-0 status/persona preconditions are not recertified.
+CH-3 2026-10-21 owner scenario: Two items1200+800 with distinct workflows. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="7" ht="190" customHeight="1">
+    <x:row r="7" ht="260" customHeight="1">
       <x:c r="A7" s="17" t="str">
         <x:v>BA-006</x:v>
       </x:c>
@@ -3684,11 +3689,12 @@
       <x:c r="N7" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">ORD-000011 and ORD-000012 item_workflow_instances present via Supabase read-only check.
-CH-2 2026-10-21: Two independent workflow instances / four stage rows verified after actual UI create. See docs_chat/CH2_BOUTIQUE_QA.md BA-006. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+CH-2 2026-10-21: Two independent workflow instances / four stage rows verified after actual UI create. See docs_chat/CH2_BOUTIQUE_QA.md BA-006. Historical V2-0 status/persona preconditions are not recertified.
+CH-3 2026-10-21 owner scenario: Two independent workflow instances/four stages persist. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="8" ht="190" customHeight="1">
+    <x:row r="8" ht="260" customHeight="1">
       <x:c r="A8" s="17" t="str">
         <x:v>BA-007</x:v>
       </x:c>
@@ -3731,11 +3737,12 @@
       <x:c r="N8" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Workflow page showed only allowed worker Designer for Design; history recorded stage started.
-CH-2 2026-10-21: Owner scenario: started QA prepare using Synthetic QA worker and QA workgroup. See docs_chat/CH2_BOUTIQUE_QA.md BA-007. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+CH-2 2026-10-21: Owner scenario: started QA prepare using Synthetic QA worker and QA workgroup. See docs_chat/CH2_BOUTIQUE_QA.md BA-007. Historical V2-0 status/persona preconditions are not recertified.
+CH-3 2026-10-21 owner scenario: Started first QA prepare with Synthetic QA worker/QA workgroup. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="9" ht="190" customHeight="1">
+    <x:row r="9" ht="260" customHeight="1">
       <x:c r="A9" s="17" t="str">
         <x:v>BA-008</x:v>
       </x:c>
@@ -3778,11 +3785,12 @@
       <x:c r="N9" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Workflow page showed item in production, 1/5 stages complete, Cutting ready_to_start.
-CH-2 2026-10-21: Completed first stage in UI; next stage ready; other item unchanged. See docs_chat/CH2_BOUTIQUE_QA.md BA-008. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+CH-2 2026-10-21: Completed first stage in UI; next stage ready; other item unchanged. See docs_chat/CH2_BOUTIQUE_QA.md BA-008. Historical V2-0 status/persona preconditions are not recertified.
+CH-3 2026-10-21 owner scenario: Completed first stage; QA finish ready, second item unchanged. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="10" ht="190" customHeight="1">
+    <x:row r="10" ht="260" customHeight="1">
       <x:c r="A10" s="17" t="str">
         <x:v>BA-009</x:v>
       </x:c>
@@ -3825,11 +3833,12 @@
       <x:c r="N10" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Tracking /track/TILaKurOoqN2o_dzXhSKK-cbmZkTos5D showed ORD-000011 and item status without internal worker data.
-CH-2 2026-10-21: Public tracking page rendered safe order/item status without internal worker, stage, payment or notes. Browser retained login; no fresh anonymous browser claim. See docs_chat/CH2_BOUTIQUE_QA.md BA-009. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+CH-2 2026-10-21: Public tracking page rendered safe order/item status without internal worker, stage, payment or notes. Browser retained login; no fresh anonymous browser claim. See docs_chat/CH2_BOUTIQUE_QA.md BA-009. Historical V2-0 status/persona preconditions are not recertified.
+CH-3 2026-10-21 owner scenario: Safe tracking shows public status only; authenticated browser, no fresh anonymous browser claim. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="11" ht="190" customHeight="1">
+    <x:row r="11" ht="260" customHeight="1">
       <x:c r="A11" s="17" t="str">
         <x:v>BA-010</x:v>
       </x:c>
@@ -3872,11 +3881,12 @@
       <x:c r="N11" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">ORD-000011 amount_paid 200, partially_paid; ORD-000012 amount_paid 300, partially_paid.
-CH-2 2026-10-21: Owner scenario: one synthetic partial receipt 300, balance 1700; no money moved. See docs_chat/CH2_BOUTIQUE_QA.md BA-010. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+CH-2 2026-10-21: Owner scenario: one synthetic partial receipt 300, balance 1700; no money moved. See docs_chat/CH2_BOUTIQUE_QA.md BA-010. Historical V2-0 status/persona preconditions are not recertified.
+CH-3 2026-10-21 owner scenario: Exactly one synthetic receipt300; balance1700, no money moved. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="12" ht="190" customHeight="1">
+    <x:row r="12" ht="260" customHeight="1">
       <x:c r="A12" s="17" t="str">
         <x:v>BA-011</x:v>
       </x:c>
@@ -3919,11 +3929,12 @@
       <x:c r="N12" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Finance GST page showed Cash in 200 for MTD and ORD-000011 receivable/payment summary.
-CH-2 2026-10-21: Owner scenario: Finance showed order collection 300 and receivable 1700. Independent Finance-role session not tested. See docs_chat/CH2_BOUTIQUE_QA.md BA-011. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+CH-2 2026-10-21: Owner scenario: Finance showed order collection 300 and receivable 1700. Independent Finance-role session not tested. See docs_chat/CH2_BOUTIQUE_QA.md BA-011. Historical V2-0 status/persona preconditions are not recertified.
+CH-3 2026-10-21 owner scenario: Finance shows ORD-000003 collection300/balance1700; aggregate cash850 includes earlier fixtures. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="13" ht="190" customHeight="1">
+    <x:row r="13" ht="260" customHeight="1">
       <x:c r="A13" s="17" t="str">
         <x:v>BA-012</x:v>
       </x:c>
@@ -3966,11 +3977,12 @@
       <x:c r="N13" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Finance GST page showed Output GST 180 and ORD-000011 in output GST list; XLSX export link present.
-CH-2 2026-10-21: Owner scenario: GST report loaded and included non-GST order when selected. Zero-GST local fixture only: GST-bearing calculation, export and filing NOT tested. See docs_chat/CH2_BOUTIQUE_QA.md BA-012. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+CH-2 2026-10-21: Owner scenario: GST report loaded and included non-GST order when selected. Zero-GST local fixture only: GST-bearing calculation, export and filing NOT tested. See docs_chat/CH2_BOUTIQUE_QA.md BA-012. Historical V2-0 status/persona preconditions are not recertified.
+CH-3 2026-10-21 owner scenario: GST report loads and includes non-GST ORD-000003. No GST-bearing calculation/export/filing claim. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="14" ht="190" customHeight="1">
+    <x:row r="14" ht="260" customHeight="1">
       <x:c r="A14" s="17" t="str">
         <x:v>BA-013</x:v>
       </x:c>
@@ -4013,11 +4025,12 @@
       <x:c r="N14" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">communication_message_queue a2b4882e-e3b6-4616-bc2b-a57acc4ae030; log 8ebc4c2f-d2f2-48a5-8454-3620b8d43cdd; no live send.
-CH-2 2026-10-21: Owner scenario: UI queued email tracking dry-run to ch2-qa@example.invalid; database dryRun=true and audit verified. No message delivered. See docs_chat/CH2_BOUTIQUE_QA.md BA-013. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+CH-2 2026-10-21: Owner scenario: UI queued email tracking dry-run to ch2-qa@example.invalid; database dryRun=true and audit verified. No message delivered. See docs_chat/CH2_BOUTIQUE_QA.md BA-013. Historical V2-0 status/persona preconditions are not recertified.
+CH-3 2026-10-21 owner scenario: Tracking email queued dry-run to ch3-qa@example.invalid; persisted dryRun/audit. No delivery. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="15" ht="190" customHeight="1">
+    <x:row r="15" ht="260" customHeight="1">
       <x:c r="A15" s="17" t="str">
         <x:v>BA-014</x:v>
       </x:c>
@@ -4060,7 +4073,8 @@
       <x:c r="N15" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">ORD-000012 notes updated to include "Edit smoke passed" without recalculating finance/production history.
-CH-2 2026-10-21: Owner scenario: edited order notes and reopened detail, total/payment/workflow preserved. See docs_chat/CH2_BOUTIQUE_QA.md BA-014. Historical V2-0 status/persona preconditions are not recertified.</x:t>
+CH-2 2026-10-21: Owner scenario: edited order notes and reopened detail, total/payment/workflow preserved. See docs_chat/CH2_BOUTIQUE_QA.md BA-014. Historical V2-0 status/persona preconditions are not recertified.
+CH-3 2026-10-21 owner scenario: Edited notes; total/payment/fit/workflows preserved. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Chat CH-4: add tenant Leads workspace and Chatwoot card
</commit_message>
<xml_diff>
--- a/docs_v2/OS_PLUS_V2_QA_Test_Matrix.xlsx
+++ b/docs_v2/OS_PLUS_V2_QA_Test_Matrix.xlsx
@@ -3406,7 +3406,7 @@
         <x:v>Evidence / Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="260" customHeight="1">
+    <x:row r="2" ht="340" customHeight="1">
       <x:c r="A2" s="17" t="str">
         <x:v>BA-001</x:v>
       </x:c>
@@ -3450,11 +3450,12 @@
         <x:is>
           <x:t xml:space="preserve">Browser: localhost:3000/dashboard; Tenant Phantom Threads; role Owner/Admin.
 CH-2 2026-10-21: Owner-a existing authenticated session and tenant selector -&gt; Local QA A verified; fresh Clerk credential entry not repeated. See docs_chat/CH2_BOUTIQUE_QA.md BA-001. Historical V2-0 status/persona preconditions are not recertified.
-CH-3 2026-10-21 owner scenario: Existing owner-a Clerk session; switched A to B and back. B cannot open new A order (404). See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
+CH-3 2026-10-21 owner scenario: Existing owner-a Clerk session; switched A to B and back. B cannot open new A order (404). See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
+CH-4 2026-10-22 owner scenario: Existing owner-a Clerk session. Actual A to B to A selection and B copied A lead/order denial. No new credential entry. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="3" ht="260" customHeight="1">
+    <x:row r="3" ht="340" customHeight="1">
       <x:c r="A3" s="17" t="str">
         <x:v>BA-002</x:v>
       </x:c>
@@ -3498,11 +3499,12 @@
         <x:is>
           <x:t xml:space="preserve">Customer ID bce5cbcb-c562-46c3-b960-e3204ab61a0f; phone search 9000000705 returned customer.
 CH-2 2026-10-21: Owner scenario: created CH2 Regression Customer and exact name search returned one match. Independent Manager session not tested. See docs_chat/CH2_BOUTIQUE_QA.md BA-002. Historical V2-0 status/persona preconditions are not recertified.
-CH-3 2026-10-21 owner scenario: Created CH3 Regression Customer; exact-name search returns one result. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
+CH-3 2026-10-21 owner scenario: Created CH3 Regression Customer; exact-name search returns one result. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
+CH-4 2026-10-22 owner scenario: Created CH4 Boutique Regression Customer using native Customers form. Exact-name search returns one result. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="4" ht="260" customHeight="1">
+    <x:row r="4" ht="340" customHeight="1">
       <x:c r="A4" s="17" t="str">
         <x:v>BA-003</x:v>
       </x:c>
@@ -3546,11 +3548,12 @@
         <x:is>
           <x:t xml:space="preserve">Measurement ID 5c2462b5-ad77-4c7b-9d81-b79db903b0d9; Chest 40, Length 28; default=true.
 CH-2 2026-10-21: Owner scenario: saved and selected garment measurement Chest 37 for both items. Dialog stays open after save, persistence passes. See docs_chat/CH2_BOUTIQUE_QA.md BA-003. Historical V2-0 status/persona preconditions are not recertified.
-CH-3 2026-10-21 owner scenario: Saved default CH3 garment fit Chest38; selected on both items. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
+CH-3 2026-10-21 owner scenario: Saved default CH3 garment fit Chest38; selected on both items. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
+CH-4 2026-10-22 owner scenario: Saved default CH4 garment fit, QA garment, Chest38. Selected and retained on both production items. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="5" ht="260" customHeight="1">
+    <x:row r="5" ht="340" customHeight="1">
       <x:c r="A5" s="17" t="str">
         <x:v>BA-004</x:v>
       </x:c>
@@ -3594,11 +3597,12 @@
         <x:is>
           <x:t xml:space="preserve">ORD-000011 / order 2d61e296-5cbd-4ca1-9d80-40c4da6bb7aa; item 52fb87ae-3604-48c4-8480-ac76dafb25b8.
 CH-2 2026-10-21: Owner scenario: created ORD-000002 / CHAT-CH2-BROWSER-QA, total 2000. See docs_chat/CH2_BOUTIQUE_QA.md BA-004. Historical V2-0 status/persona preconditions are not recertified.
-CH-3 2026-10-21 owner scenario: Created ORD-000003 / CHAT-CH3-BROWSER-QA total2000. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
+CH-3 2026-10-21 owner scenario: Created ORD-000003 / CHAT-CH3-BROWSER-QA total2000. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
+CH-4 2026-10-22 owner scenario: Created ORD-000004 / CHAT-CH4-BROWSER-QA, total2000. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="6" ht="260" customHeight="1">
+    <x:row r="6" ht="340" customHeight="1">
       <x:c r="A6" s="17" t="str">
         <x:v>BA-005</x:v>
       </x:c>
@@ -3642,11 +3646,12 @@
         <x:is>
           <x:t xml:space="preserve">ORD-000012 / order 3b27cca4-6796-46cb-b157-0890d109a4ee; two order_items with Default and Painting 1 workflow IDs.
 CH-2 2026-10-21: Owner scenario: two items 1200 + 800, each with a different workflow. See docs_chat/CH2_BOUTIQUE_QA.md BA-005. Historical V2-0 status/persona preconditions are not recertified.
-CH-3 2026-10-21 owner scenario: Two items1200+800 with distinct workflows. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
+CH-3 2026-10-21 owner scenario: Two items1200+800 with distinct workflows. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
+CH-4 2026-10-22 owner scenario: Two items1200 and800 with distinct existing workflows. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="7" ht="260" customHeight="1">
+    <x:row r="7" ht="340" customHeight="1">
       <x:c r="A7" s="17" t="str">
         <x:v>BA-006</x:v>
       </x:c>
@@ -3690,11 +3695,12 @@
         <x:is>
           <x:t xml:space="preserve">ORD-000011 and ORD-000012 item_workflow_instances present via Supabase read-only check.
 CH-2 2026-10-21: Two independent workflow instances / four stage rows verified after actual UI create. See docs_chat/CH2_BOUTIQUE_QA.md BA-006. Historical V2-0 status/persona preconditions are not recertified.
-CH-3 2026-10-21 owner scenario: Two independent workflow instances/four stages persist. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
+CH-3 2026-10-21 owner scenario: Two independent workflow instances/four stages persist. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
+CH-4 2026-10-22 owner scenario: Two independent workflow instances and four stages persisted. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="8" ht="260" customHeight="1">
+    <x:row r="8" ht="340" customHeight="1">
       <x:c r="A8" s="17" t="str">
         <x:v>BA-007</x:v>
       </x:c>
@@ -3738,11 +3744,12 @@
         <x:is>
           <x:t xml:space="preserve">Workflow page showed only allowed worker Designer for Design; history recorded stage started.
 CH-2 2026-10-21: Owner scenario: started QA prepare using Synthetic QA worker and QA workgroup. See docs_chat/CH2_BOUTIQUE_QA.md BA-007. Historical V2-0 status/persona preconditions are not recertified.
-CH-3 2026-10-21 owner scenario: Started first QA prepare with Synthetic QA worker/QA workgroup. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
+CH-3 2026-10-21 owner scenario: Started first QA prepare with Synthetic QA worker/QA workgroup. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
+CH-4 2026-10-22 owner scenario: Started QA prepare with Synthetic QA worker and eligible QA workgroup. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="9" ht="260" customHeight="1">
+    <x:row r="9" ht="340" customHeight="1">
       <x:c r="A9" s="17" t="str">
         <x:v>BA-008</x:v>
       </x:c>
@@ -3786,11 +3793,12 @@
         <x:is>
           <x:t xml:space="preserve">Workflow page showed item in production, 1/5 stages complete, Cutting ready_to_start.
 CH-2 2026-10-21: Completed first stage in UI; next stage ready; other item unchanged. See docs_chat/CH2_BOUTIQUE_QA.md BA-008. Historical V2-0 status/persona preconditions are not recertified.
-CH-3 2026-10-21 owner scenario: Completed first stage; QA finish ready, second item unchanged. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
+CH-3 2026-10-21 owner scenario: Completed first stage; QA finish ready, second item unchanged. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
+CH-4 2026-10-22 owner scenario: Completed top first stage. QA finish is ready. Skirt unchanged. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="10" ht="260" customHeight="1">
+    <x:row r="10" ht="340" customHeight="1">
       <x:c r="A10" s="17" t="str">
         <x:v>BA-009</x:v>
       </x:c>
@@ -3834,11 +3842,12 @@
         <x:is>
           <x:t xml:space="preserve">Tracking /track/TILaKurOoqN2o_dzXhSKK-cbmZkTos5D showed ORD-000011 and item status without internal worker data.
 CH-2 2026-10-21: Public tracking page rendered safe order/item status without internal worker, stage, payment or notes. Browser retained login; no fresh anonymous browser claim. See docs_chat/CH2_BOUTIQUE_QA.md BA-009. Historical V2-0 status/persona preconditions are not recertified.
-CH-3 2026-10-21 owner scenario: Safe tracking shows public status only; authenticated browser, no fresh anonymous browser claim. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
+CH-3 2026-10-21 owner scenario: Safe tracking shows public status only; authenticated browser, no fresh anonymous browser claim. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
+CH-4 2026-10-22 owner scenario: Tracking browser and separate anonymous HTTP200 expose public status without internal stages, worker, notes, receipt reference or email. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="11" ht="260" customHeight="1">
+    <x:row r="11" ht="340" customHeight="1">
       <x:c r="A11" s="17" t="str">
         <x:v>BA-010</x:v>
       </x:c>
@@ -3882,11 +3891,12 @@
         <x:is>
           <x:t xml:space="preserve">ORD-000011 amount_paid 200, partially_paid; ORD-000012 amount_paid 300, partially_paid.
 CH-2 2026-10-21: Owner scenario: one synthetic partial receipt 300, balance 1700; no money moved. See docs_chat/CH2_BOUTIQUE_QA.md BA-010. Historical V2-0 status/persona preconditions are not recertified.
-CH-3 2026-10-21 owner scenario: Exactly one synthetic receipt300; balance1700, no money moved. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
+CH-3 2026-10-21 owner scenario: Exactly one synthetic receipt300; balance1700, no money moved. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
+CH-4 2026-10-22 owner scenario: Exactly one synthetic receipt300. Balance1700. No money moved. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="12" ht="260" customHeight="1">
+    <x:row r="12" ht="340" customHeight="1">
       <x:c r="A12" s="17" t="str">
         <x:v>BA-011</x:v>
       </x:c>
@@ -3930,11 +3940,12 @@
         <x:is>
           <x:t xml:space="preserve">Finance GST page showed Cash in 200 for MTD and ORD-000011 receivable/payment summary.
 CH-2 2026-10-21: Owner scenario: Finance showed order collection 300 and receivable 1700. Independent Finance-role session not tested. See docs_chat/CH2_BOUTIQUE_QA.md BA-011. Historical V2-0 status/persona preconditions are not recertified.
-CH-3 2026-10-21 owner scenario: Finance shows ORD-000003 collection300/balance1700; aggregate cash850 includes earlier fixtures. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
+CH-3 2026-10-21 owner scenario: Finance shows ORD-000003 collection300/balance1700; aggregate cash850 includes earlier fixtures. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
+CH-4 2026-10-22 owner scenario: Finance shows ORD-000004 collection300 and balance1700. Aggregate1150 includes earlier local receipts. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="13" ht="260" customHeight="1">
+    <x:row r="13" ht="340" customHeight="1">
       <x:c r="A13" s="17" t="str">
         <x:v>BA-012</x:v>
       </x:c>
@@ -3978,11 +3989,12 @@
         <x:is>
           <x:t xml:space="preserve">Finance GST page showed Output GST 180 and ORD-000011 in output GST list; XLSX export link present.
 CH-2 2026-10-21: Owner scenario: GST report loaded and included non-GST order when selected. Zero-GST local fixture only: GST-bearing calculation, export and filing NOT tested. See docs_chat/CH2_BOUTIQUE_QA.md BA-012. Historical V2-0 status/persona preconditions are not recertified.
-CH-3 2026-10-21 owner scenario: GST report loads and includes non-GST ORD-000003. No GST-bearing calculation/export/filing claim. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
+CH-3 2026-10-21 owner scenario: GST report loads and includes non-GST ORD-000003. No GST-bearing calculation/export/filing claim. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
+CH-4 2026-10-22 owner scenario: GST report loads with the non-GST test order. No GST-bearing calculation, export or filing acceptance. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="14" ht="260" customHeight="1">
+    <x:row r="14" ht="340" customHeight="1">
       <x:c r="A14" s="17" t="str">
         <x:v>BA-013</x:v>
       </x:c>
@@ -4026,11 +4038,12 @@
         <x:is>
           <x:t xml:space="preserve">communication_message_queue a2b4882e-e3b6-4616-bc2b-a57acc4ae030; log 8ebc4c2f-d2f2-48a5-8454-3620b8d43cdd; no live send.
 CH-2 2026-10-21: Owner scenario: UI queued email tracking dry-run to ch2-qa@example.invalid; database dryRun=true and audit verified. No message delivered. See docs_chat/CH2_BOUTIQUE_QA.md BA-013. Historical V2-0 status/persona preconditions are not recertified.
-CH-3 2026-10-21 owner scenario: Tracking email queued dry-run to ch3-qa@example.invalid; persisted dryRun/audit. No delivery. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
+CH-3 2026-10-21 owner scenario: Tracking email queued dry-run to ch3-qa@example.invalid; persisted dryRun/audit. No delivery. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
+CH-4 2026-10-22 owner scenario: Tracking email queued only as dry-run to ch4-qa@example.invalid. Dry-run flag and audit persisted. No delivery. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="15" ht="260" customHeight="1">
+    <x:row r="15" ht="340" customHeight="1">
       <x:c r="A15" s="17" t="str">
         <x:v>BA-014</x:v>
       </x:c>
@@ -4074,7 +4087,8 @@
         <x:is>
           <x:t xml:space="preserve">ORD-000012 notes updated to include "Edit smoke passed" without recalculating finance/production history.
 CH-2 2026-10-21: Owner scenario: edited order notes and reopened detail, total/payment/workflow preserved. See docs_chat/CH2_BOUTIQUE_QA.md BA-014. Historical V2-0 status/persona preconditions are not recertified.
-CH-3 2026-10-21 owner scenario: Edited notes; total/payment/fit/workflows preserved. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.</x:t>
+CH-3 2026-10-21 owner scenario: Edited notes; total/payment/fit/workflows preserved. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
+CH-4 2026-10-22 owner scenario: Edited notes. Payment, totals, measurements and workflow history preserved. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Chat CH-5: guarded mock drafts and native reply workflow
</commit_message>
<xml_diff>
--- a/docs_v2/OS_PLUS_V2_QA_Test_Matrix.xlsx
+++ b/docs_v2/OS_PLUS_V2_QA_Test_Matrix.xlsx
@@ -3406,7 +3406,7 @@
         <x:v>Evidence / Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="340" customHeight="1">
+    <x:row r="2" ht="409.5" customHeight="1">
       <x:c r="A2" s="17" t="str">
         <x:v>BA-001</x:v>
       </x:c>
@@ -3451,11 +3451,12 @@
           <x:t xml:space="preserve">Browser: localhost:3000/dashboard; Tenant Phantom Threads; role Owner/Admin.
 CH-2 2026-10-21: Owner-a existing authenticated session and tenant selector -&gt; Local QA A verified; fresh Clerk credential entry not repeated. See docs_chat/CH2_BOUTIQUE_QA.md BA-001. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Existing owner-a Clerk session; switched A to B and back. B cannot open new A order (404). See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
-CH-4 2026-10-22 owner scenario: Existing owner-a Clerk session. Actual A to B to A selection and B copied A lead/order denial. No new credential entry. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
+CH-4 2026-10-22 owner scenario: Existing owner-a Clerk session. Actual A to B to A selection and B copied A lead/order denial. No new credential entry. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
+CH-5 2026-10-22 owner scenario: Existing owner-a Clerk session. Actual A to B to A selection and B copied A lead/order denial. No new credential entry. See docs_chat/CH5_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="3" ht="340" customHeight="1">
+    <x:row r="3" ht="409.5" customHeight="1">
       <x:c r="A3" s="17" t="str">
         <x:v>BA-002</x:v>
       </x:c>
@@ -3500,11 +3501,12 @@
           <x:t xml:space="preserve">Customer ID bce5cbcb-c562-46c3-b960-e3204ab61a0f; phone search 9000000705 returned customer.
 CH-2 2026-10-21: Owner scenario: created CH2 Regression Customer and exact name search returned one match. Independent Manager session not tested. See docs_chat/CH2_BOUTIQUE_QA.md BA-002. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Created CH3 Regression Customer; exact-name search returns one result. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
-CH-4 2026-10-22 owner scenario: Created CH4 Boutique Regression Customer using native Customers form. Exact-name search returns one result. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
+CH-4 2026-10-22 owner scenario: Created CH4 Boutique Regression Customer using native Customers form. Exact-name search returns one result. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
+CH-5 2026-10-22 owner scenario: Created CH5 Boutique Regression Customer using native Customers form. Exact-name search returns one result. See docs_chat/CH5_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="4" ht="340" customHeight="1">
+    <x:row r="4" ht="409.5" customHeight="1">
       <x:c r="A4" s="17" t="str">
         <x:v>BA-003</x:v>
       </x:c>
@@ -3549,11 +3551,12 @@
           <x:t xml:space="preserve">Measurement ID 5c2462b5-ad77-4c7b-9d81-b79db903b0d9; Chest 40, Length 28; default=true.
 CH-2 2026-10-21: Owner scenario: saved and selected garment measurement Chest 37 for both items. Dialog stays open after save, persistence passes. See docs_chat/CH2_BOUTIQUE_QA.md BA-003. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Saved default CH3 garment fit Chest38; selected on both items. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
-CH-4 2026-10-22 owner scenario: Saved default CH4 garment fit, QA garment, Chest38. Selected and retained on both production items. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
+CH-4 2026-10-22 owner scenario: Saved default CH4 garment fit, QA garment, Chest38. Selected and retained on both production items. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
+CH-5 2026-10-22 owner scenario: Saved default CH5 garment fit, QA garment, Chest38. Selected and retained on both production items. See docs_chat/CH5_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="5" ht="340" customHeight="1">
+    <x:row r="5" ht="409.5" customHeight="1">
       <x:c r="A5" s="17" t="str">
         <x:v>BA-004</x:v>
       </x:c>
@@ -3598,11 +3601,12 @@
           <x:t xml:space="preserve">ORD-000011 / order 2d61e296-5cbd-4ca1-9d80-40c4da6bb7aa; item 52fb87ae-3604-48c4-8480-ac76dafb25b8.
 CH-2 2026-10-21: Owner scenario: created ORD-000002 / CHAT-CH2-BROWSER-QA, total 2000. See docs_chat/CH2_BOUTIQUE_QA.md BA-004. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Created ORD-000003 / CHAT-CH3-BROWSER-QA total2000. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
-CH-4 2026-10-22 owner scenario: Created ORD-000004 / CHAT-CH4-BROWSER-QA, total2000. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
+CH-4 2026-10-22 owner scenario: Created ORD-000004 / CHAT-CH4-BROWSER-QA, total2000. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
+CH-5 2026-10-22 owner scenario: Created ORD-000005 / CHAT-CH5-BROWSER-QA, total2000. See docs_chat/CH5_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="6" ht="340" customHeight="1">
+    <x:row r="6" ht="409.5" customHeight="1">
       <x:c r="A6" s="17" t="str">
         <x:v>BA-005</x:v>
       </x:c>
@@ -3647,11 +3651,12 @@
           <x:t xml:space="preserve">ORD-000012 / order 3b27cca4-6796-46cb-b157-0890d109a4ee; two order_items with Default and Painting 1 workflow IDs.
 CH-2 2026-10-21: Owner scenario: two items 1200 + 800, each with a different workflow. See docs_chat/CH2_BOUTIQUE_QA.md BA-005. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Two items1200+800 with distinct workflows. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
-CH-4 2026-10-22 owner scenario: Two items1200 and800 with distinct existing workflows. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
+CH-4 2026-10-22 owner scenario: Two items1200 and800 with distinct existing workflows. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
+CH-5 2026-10-22 owner scenario: Two items1200 and800 with distinct existing workflows. See docs_chat/CH5_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="7" ht="340" customHeight="1">
+    <x:row r="7" ht="409.5" customHeight="1">
       <x:c r="A7" s="17" t="str">
         <x:v>BA-006</x:v>
       </x:c>
@@ -3696,11 +3701,12 @@
           <x:t xml:space="preserve">ORD-000011 and ORD-000012 item_workflow_instances present via Supabase read-only check.
 CH-2 2026-10-21: Two independent workflow instances / four stage rows verified after actual UI create. See docs_chat/CH2_BOUTIQUE_QA.md BA-006. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Two independent workflow instances/four stages persist. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
-CH-4 2026-10-22 owner scenario: Two independent workflow instances and four stages persisted. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
+CH-4 2026-10-22 owner scenario: Two independent workflow instances and four stages persisted. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
+CH-5 2026-10-22 owner scenario: Two independent workflow instances and four stages persisted. See docs_chat/CH5_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="8" ht="340" customHeight="1">
+    <x:row r="8" ht="409.5" customHeight="1">
       <x:c r="A8" s="17" t="str">
         <x:v>BA-007</x:v>
       </x:c>
@@ -3745,11 +3751,12 @@
           <x:t xml:space="preserve">Workflow page showed only allowed worker Designer for Design; history recorded stage started.
 CH-2 2026-10-21: Owner scenario: started QA prepare using Synthetic QA worker and QA workgroup. See docs_chat/CH2_BOUTIQUE_QA.md BA-007. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Started first QA prepare with Synthetic QA worker/QA workgroup. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
-CH-4 2026-10-22 owner scenario: Started QA prepare with Synthetic QA worker and eligible QA workgroup. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
+CH-4 2026-10-22 owner scenario: Started QA prepare with Synthetic QA worker and eligible QA workgroup. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
+CH-5 2026-10-22 owner scenario: Started QA prepare with Synthetic QA worker and eligible QA workgroup. See docs_chat/CH5_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="9" ht="340" customHeight="1">
+    <x:row r="9" ht="409.5" customHeight="1">
       <x:c r="A9" s="17" t="str">
         <x:v>BA-008</x:v>
       </x:c>
@@ -3794,11 +3801,12 @@
           <x:t xml:space="preserve">Workflow page showed item in production, 1/5 stages complete, Cutting ready_to_start.
 CH-2 2026-10-21: Completed first stage in UI; next stage ready; other item unchanged. See docs_chat/CH2_BOUTIQUE_QA.md BA-008. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Completed first stage; QA finish ready, second item unchanged. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
-CH-4 2026-10-22 owner scenario: Completed top first stage. QA finish is ready. Skirt unchanged. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
+CH-4 2026-10-22 owner scenario: Completed top first stage. QA finish is ready. Skirt unchanged. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
+CH-5 2026-10-22 owner scenario: Completed top first stage. QA finish is ready. Skirt unchanged. See docs_chat/CH5_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="10" ht="340" customHeight="1">
+    <x:row r="10" ht="409.5" customHeight="1">
       <x:c r="A10" s="17" t="str">
         <x:v>BA-009</x:v>
       </x:c>
@@ -3843,11 +3851,12 @@
           <x:t xml:space="preserve">Tracking /track/TILaKurOoqN2o_dzXhSKK-cbmZkTos5D showed ORD-000011 and item status without internal worker data.
 CH-2 2026-10-21: Public tracking page rendered safe order/item status without internal worker, stage, payment or notes. Browser retained login; no fresh anonymous browser claim. See docs_chat/CH2_BOUTIQUE_QA.md BA-009. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Safe tracking shows public status only; authenticated browser, no fresh anonymous browser claim. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
-CH-4 2026-10-22 owner scenario: Tracking browser and separate anonymous HTTP200 expose public status without internal stages, worker, notes, receipt reference or email. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
+CH-4 2026-10-22 owner scenario: Tracking browser and separate anonymous HTTP200 expose public status without internal stages, worker, notes, receipt reference or email. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
+CH-5 2026-10-22 owner scenario: Tracking browser and separate anonymous HTTP200 expose public status without internal stages, worker, notes, receipt reference or email. See docs_chat/CH5_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="11" ht="340" customHeight="1">
+    <x:row r="11" ht="409.5" customHeight="1">
       <x:c r="A11" s="17" t="str">
         <x:v>BA-010</x:v>
       </x:c>
@@ -3892,11 +3901,12 @@
           <x:t xml:space="preserve">ORD-000011 amount_paid 200, partially_paid; ORD-000012 amount_paid 300, partially_paid.
 CH-2 2026-10-21: Owner scenario: one synthetic partial receipt 300, balance 1700; no money moved. See docs_chat/CH2_BOUTIQUE_QA.md BA-010. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Exactly one synthetic receipt300; balance1700, no money moved. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
-CH-4 2026-10-22 owner scenario: Exactly one synthetic receipt300. Balance1700. No money moved. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
+CH-4 2026-10-22 owner scenario: Exactly one synthetic receipt300. Balance1700. No money moved. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
+CH-5 2026-10-22 owner scenario: Exactly one synthetic receipt300. Balance1700. No money moved. See docs_chat/CH5_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="12" ht="340" customHeight="1">
+    <x:row r="12" ht="409.5" customHeight="1">
       <x:c r="A12" s="17" t="str">
         <x:v>BA-011</x:v>
       </x:c>
@@ -3941,11 +3951,12 @@
           <x:t xml:space="preserve">Finance GST page showed Cash in 200 for MTD and ORD-000011 receivable/payment summary.
 CH-2 2026-10-21: Owner scenario: Finance showed order collection 300 and receivable 1700. Independent Finance-role session not tested. See docs_chat/CH2_BOUTIQUE_QA.md BA-011. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Finance shows ORD-000003 collection300/balance1700; aggregate cash850 includes earlier fixtures. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
-CH-4 2026-10-22 owner scenario: Finance shows ORD-000004 collection300 and balance1700. Aggregate1150 includes earlier local receipts. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
+CH-4 2026-10-22 owner scenario: Finance shows ORD-000004 collection300 and balance1700. Aggregate1150 includes earlier local receipts. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
+CH-5 2026-10-22 owner scenario: Finance shows ORD-000005 collection300 and balance1700. Aggregate1450 includes earlier local receipts. See docs_chat/CH5_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="13" ht="340" customHeight="1">
+    <x:row r="13" ht="409.5" customHeight="1">
       <x:c r="A13" s="17" t="str">
         <x:v>BA-012</x:v>
       </x:c>
@@ -3990,11 +4001,12 @@
           <x:t xml:space="preserve">Finance GST page showed Output GST 180 and ORD-000011 in output GST list; XLSX export link present.
 CH-2 2026-10-21: Owner scenario: GST report loaded and included non-GST order when selected. Zero-GST local fixture only: GST-bearing calculation, export and filing NOT tested. See docs_chat/CH2_BOUTIQUE_QA.md BA-012. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: GST report loads and includes non-GST ORD-000003. No GST-bearing calculation/export/filing claim. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
-CH-4 2026-10-22 owner scenario: GST report loads with the non-GST test order. No GST-bearing calculation, export or filing acceptance. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
+CH-4 2026-10-22 owner scenario: GST report loads with the non-GST test order. No GST-bearing calculation, export or filing acceptance. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
+CH-5 2026-10-22 owner scenario: GST report loads with the non-GST test order. No GST-bearing calculation, export or filing acceptance. See docs_chat/CH5_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="14" ht="340" customHeight="1">
+    <x:row r="14" ht="409.5" customHeight="1">
       <x:c r="A14" s="17" t="str">
         <x:v>BA-013</x:v>
       </x:c>
@@ -4039,11 +4051,12 @@
           <x:t xml:space="preserve">communication_message_queue a2b4882e-e3b6-4616-bc2b-a57acc4ae030; log 8ebc4c2f-d2f2-48a5-8454-3620b8d43cdd; no live send.
 CH-2 2026-10-21: Owner scenario: UI queued email tracking dry-run to ch2-qa@example.invalid; database dryRun=true and audit verified. No message delivered. See docs_chat/CH2_BOUTIQUE_QA.md BA-013. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Tracking email queued dry-run to ch3-qa@example.invalid; persisted dryRun/audit. No delivery. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
-CH-4 2026-10-22 owner scenario: Tracking email queued only as dry-run to ch4-qa@example.invalid. Dry-run flag and audit persisted. No delivery. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
+CH-4 2026-10-22 owner scenario: Tracking email queued only as dry-run to ch4-qa@example.invalid. Dry-run flag and audit persisted. No delivery. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
+CH-5 2026-10-22 owner scenario: Tracking email queued only as dry-run to ch5-qa@example.invalid. Dry-run flag and audit persisted. No delivery. See docs_chat/CH5_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="15" ht="340" customHeight="1">
+    <x:row r="15" ht="409.5" customHeight="1">
       <x:c r="A15" s="17" t="str">
         <x:v>BA-014</x:v>
       </x:c>
@@ -4088,7 +4101,8 @@
           <x:t xml:space="preserve">ORD-000012 notes updated to include "Edit smoke passed" without recalculating finance/production history.
 CH-2 2026-10-21: Owner scenario: edited order notes and reopened detail, total/payment/workflow preserved. See docs_chat/CH2_BOUTIQUE_QA.md BA-014. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Edited notes; total/payment/fit/workflows preserved. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
-CH-4 2026-10-22 owner scenario: Edited notes. Payment, totals, measurements and workflow history preserved. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
+CH-4 2026-10-22 owner scenario: Edited notes. Payment, totals, measurements and workflow history preserved. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
+CH-5 2026-10-22 owner scenario: Edited notes. Payment, totals, measurements and workflow history preserved. See docs_chat/CH5_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Chat CH-6: add guarded requests, handoffs and local auto actions
</commit_message>
<xml_diff>
--- a/docs_v2/OS_PLUS_V2_QA_Test_Matrix.xlsx
+++ b/docs_v2/OS_PLUS_V2_QA_Test_Matrix.xlsx
@@ -3359,7 +3359,7 @@
     <x:col min="11" max="11" width="14" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="32" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="38" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="68" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -3443,12 +3443,16 @@
       <x:c r="L2" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="M2" s="17" t="str">
-        <x:v>Authenticated Owner/Admin opened Phantom Threads dashboard.</x:v>
+      <x:c r="M2" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Retained owner-a Clerk session. A to B to A selection. B copied A order/customer/lead URLs return404. No fresh credential entry.</x:t>
+        </x:is>
       </x:c>
       <x:c r="N2" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Browser: localhost:3000/dashboard; Tenant Phantom Threads; role Owner/Admin.
+          <x:t xml:space="preserve">CH-6 2026-10-24 LOCAL: Retained owner-a Clerk session. A to B to A selection. B copied A order/customer/lead URLs return404. No fresh credential entry. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
+Prior actual result: Authenticated Owner/Admin opened Phantom Threads dashboard.
+Browser: localhost:3000/dashboard; Tenant Phantom Threads; role Owner/Admin.
 CH-2 2026-10-21: Owner-a existing authenticated session and tenant selector -&gt; Local QA A verified; fresh Clerk credential entry not repeated. See docs_chat/CH2_BOUTIQUE_QA.md BA-001. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Existing owner-a Clerk session; switched A to B and back. B cannot open new A order (404). See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
 CH-4 2026-10-22 owner scenario: Existing owner-a Clerk session. Actual A to B to A selection and B copied A lead/order denial. No new credential entry. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
@@ -3493,12 +3497,16 @@
       <x:c r="L3" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="M3" s="17" t="str">
-        <x:v>Created V2 QA Customer 20260705 and found it via phone suggestion.</x:v>
+      <x:c r="M3" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Native customer form created CH6 Boutique Regression Customer. Exact-name search returns one customer.</x:t>
+        </x:is>
       </x:c>
       <x:c r="N3" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Customer ID bce5cbcb-c562-46c3-b960-e3204ab61a0f; phone search 9000000705 returned customer.
+          <x:t xml:space="preserve">CH-6 2026-10-24 LOCAL: Native customer form created CH6 Boutique Regression Customer. Exact-name search returns one customer. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
+Prior actual result: Created V2 QA Customer 20260705 and found it via phone suggestion.
+Customer ID bce5cbcb-c562-46c3-b960-e3204ab61a0f; phone search 9000000705 returned customer.
 CH-2 2026-10-21: Owner scenario: created CH2 Regression Customer and exact name search returned one match. Independent Manager session not tested. See docs_chat/CH2_BOUTIQUE_QA.md BA-002. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Created CH3 Regression Customer; exact-name search returns one result. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
 CH-4 2026-10-22 owner scenario: Created CH4 Boutique Regression Customer using native Customers form. Exact-name search returns one result. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
@@ -3543,12 +3551,16 @@
       <x:c r="L4" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="M4" s="17" t="str">
-        <x:v>Created default Shirt measurement and verified order-form fit reference.</x:v>
+      <x:c r="M4" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Saved CH6 garment fit, default QA garment, Chest38. Selected on both new items.</x:t>
+        </x:is>
       </x:c>
       <x:c r="N4" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Measurement ID 5c2462b5-ad77-4c7b-9d81-b79db903b0d9; Chest 40, Length 28; default=true.
+          <x:t xml:space="preserve">CH-6 2026-10-24 LOCAL: Saved CH6 garment fit, default QA garment, Chest38. Selected on both new items. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
+Prior actual result: Created default Shirt measurement and verified order-form fit reference.
+Measurement ID 5c2462b5-ad77-4c7b-9d81-b79db903b0d9; Chest 40, Length 28; default=true.
 CH-2 2026-10-21: Owner scenario: saved and selected garment measurement Chest 37 for both items. Dialog stays open after save, persistence passes. See docs_chat/CH2_BOUTIQUE_QA.md BA-003. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Saved default CH3 garment fit Chest38; selected on both items. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
 CH-4 2026-10-22 owner scenario: Saved default CH4 garment fit, QA garment, Chest38. Selected and retained on both production items. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
@@ -3593,12 +3605,16 @@
       <x:c r="L5" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="M5" s="17" t="str">
-        <x:v>Created Boutique order with one item using legacy order_items runtime.</x:v>
+      <x:c r="M5" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Created ORD-000006, reference CHAT-CH6-BROWSER-QA, total2000.</x:t>
+        </x:is>
       </x:c>
       <x:c r="N5" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">ORD-000011 / order 2d61e296-5cbd-4ca1-9d80-40c4da6bb7aa; item 52fb87ae-3604-48c4-8480-ac76dafb25b8.
+          <x:t xml:space="preserve">CH-6 2026-10-24 LOCAL: Created ORD-000006, reference CHAT-CH6-BROWSER-QA, total2000. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
+Prior actual result: Created Boutique order with one item using legacy order_items runtime.
+ORD-000011 / order 2d61e296-5cbd-4ca1-9d80-40c4da6bb7aa; item 52fb87ae-3604-48c4-8480-ac76dafb25b8.
 CH-2 2026-10-21: Owner scenario: created ORD-000002 / CHAT-CH2-BROWSER-QA, total 2000. See docs_chat/CH2_BOUTIQUE_QA.md BA-004. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Created ORD-000003 / CHAT-CH3-BROWSER-QA total2000. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
 CH-4 2026-10-22 owner scenario: Created ORD-000004 / CHAT-CH4-BROWSER-QA, total2000. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
@@ -3643,12 +3659,16 @@
       <x:c r="L6" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="M6" s="17" t="str">
-        <x:v>Created two-item Boutique order with different workflows.</x:v>
+      <x:c r="M6" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Created CH6 top1200 and CH6 skirt800 with distinct existing workflows.</x:t>
+        </x:is>
       </x:c>
       <x:c r="N6" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">ORD-000012 / order 3b27cca4-6796-46cb-b157-0890d109a4ee; two order_items with Default and Painting 1 workflow IDs.
+          <x:t xml:space="preserve">CH-6 2026-10-24 LOCAL: Created CH6 top1200 and CH6 skirt800 with distinct existing workflows. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
+Prior actual result: Created two-item Boutique order with different workflows.
+ORD-000012 / order 3b27cca4-6796-46cb-b157-0890d109a4ee; two order_items with Default and Painting 1 workflow IDs.
 CH-2 2026-10-21: Owner scenario: two items 1200 + 800, each with a different workflow. See docs_chat/CH2_BOUTIQUE_QA.md BA-005. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Two items1200+800 with distinct workflows. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
 CH-4 2026-10-22 owner scenario: Two items1200 and800 with distinct existing workflows. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
@@ -3693,12 +3713,16 @@
       <x:c r="L7" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="M7" s="17" t="str">
-        <x:v>Verified workflow instances exist for created order items.</x:v>
+      <x:c r="M7" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Two workflow instances and four stage instances persisted.</x:t>
+        </x:is>
       </x:c>
       <x:c r="N7" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">ORD-000011 and ORD-000012 item_workflow_instances present via Supabase read-only check.
+          <x:t xml:space="preserve">CH-6 2026-10-24 LOCAL: Two workflow instances and four stage instances persisted. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
+Prior actual result: Verified workflow instances exist for created order items.
+ORD-000011 and ORD-000012 item_workflow_instances present via Supabase read-only check.
 CH-2 2026-10-21: Two independent workflow instances / four stage rows verified after actual UI create. See docs_chat/CH2_BOUTIQUE_QA.md BA-006. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Two independent workflow instances/four stages persist. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
 CH-4 2026-10-22 owner scenario: Two independent workflow instances and four stages persisted. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
@@ -3743,12 +3767,16 @@
       <x:c r="L8" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="M8" s="17" t="str">
-        <x:v>Started Design stage with allowed Designer worker.</x:v>
+      <x:c r="M8" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Started QA prepare with Synthetic QA worker and eligible QA workgroup.</x:t>
+        </x:is>
       </x:c>
       <x:c r="N8" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Workflow page showed only allowed worker Designer for Design; history recorded stage started.
+          <x:t xml:space="preserve">CH-6 2026-10-24 LOCAL: Started QA prepare with Synthetic QA worker and eligible QA workgroup. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
+Prior actual result: Started Design stage with allowed Designer worker.
+Workflow page showed only allowed worker Designer for Design; history recorded stage started.
 CH-2 2026-10-21: Owner scenario: started QA prepare using Synthetic QA worker and QA workgroup. See docs_chat/CH2_BOUTIQUE_QA.md BA-007. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Started first QA prepare with Synthetic QA worker/QA workgroup. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
 CH-4 2026-10-22 owner scenario: Started QA prepare with Synthetic QA worker and eligible QA workgroup. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
@@ -3793,12 +3821,16 @@
       <x:c r="L9" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="M9" s="17" t="str">
-        <x:v>Completed Design stage and Cutting became ready.</x:v>
+      <x:c r="M9" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Completed top first stage; QA finish ready; skirt unchanged.</x:t>
+        </x:is>
       </x:c>
       <x:c r="N9" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Workflow page showed item in production, 1/5 stages complete, Cutting ready_to_start.
+          <x:t xml:space="preserve">CH-6 2026-10-24 LOCAL: Completed top first stage; QA finish ready; skirt unchanged. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
+Prior actual result: Completed Design stage and Cutting became ready.
+Workflow page showed item in production, 1/5 stages complete, Cutting ready_to_start.
 CH-2 2026-10-21: Completed first stage in UI; next stage ready; other item unchanged. See docs_chat/CH2_BOUTIQUE_QA.md BA-008. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Completed first stage; QA finish ready, second item unchanged. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
 CH-4 2026-10-22 owner scenario: Completed top first stage. QA finish is ready. Skirt unchanged. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
@@ -3843,12 +3875,16 @@
       <x:c r="L10" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="M10" s="17" t="str">
-        <x:v>Opened public tracking link and verified customer-safe status.</x:v>
+      <x:c r="M10" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Browser public tracking plus separate anonymous HTTP200 exclude internal stages, worker, notes, receipt reference and email.</x:t>
+        </x:is>
       </x:c>
       <x:c r="N10" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Tracking /track/TILaKurOoqN2o_dzXhSKK-cbmZkTos5D showed ORD-000011 and item status without internal worker data.
+          <x:t xml:space="preserve">CH-6 2026-10-24 LOCAL: Browser public tracking plus separate anonymous HTTP200 exclude internal stages, worker, notes, receipt reference and email. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
+Prior actual result: Opened public tracking link and verified customer-safe status.
+Tracking /track/TILaKurOoqN2o_dzXhSKK-cbmZkTos5D showed ORD-000011 and item status without internal worker data.
 CH-2 2026-10-21: Public tracking page rendered safe order/item status without internal worker, stage, payment or notes. Browser retained login; no fresh anonymous browser claim. See docs_chat/CH2_BOUTIQUE_QA.md BA-009. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Safe tracking shows public status only; authenticated browser, no fresh anonymous browser claim. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
 CH-4 2026-10-22 owner scenario: Tracking browser and separate anonymous HTTP200 expose public status without internal stages, worker, notes, receipt reference or email. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
@@ -3893,12 +3929,16 @@
       <x:c r="L11" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="M11" s="17" t="str">
-        <x:v>Recorded partial payment during order creation and verified order_payments/payment status.</x:v>
+      <x:c r="M11" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Exactly one synthetic cash receipt300; remaining1700. No money moved.</x:t>
+        </x:is>
       </x:c>
       <x:c r="N11" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">ORD-000011 amount_paid 200, partially_paid; ORD-000012 amount_paid 300, partially_paid.
+          <x:t xml:space="preserve">CH-6 2026-10-24 LOCAL: Exactly one synthetic cash receipt300; remaining1700. No money moved. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
+Prior actual result: Recorded partial payment during order creation and verified order_payments/payment status.
+ORD-000011 amount_paid 200, partially_paid; ORD-000012 amount_paid 300, partially_paid.
 CH-2 2026-10-21: Owner scenario: one synthetic partial receipt 300, balance 1700; no money moved. See docs_chat/CH2_BOUTIQUE_QA.md BA-010. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Exactly one synthetic receipt300; balance1700, no money moved. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
 CH-4 2026-10-22 owner scenario: Exactly one synthetic receipt300. Balance1700. No money moved. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
@@ -3943,12 +3983,16 @@
       <x:c r="L12" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="M12" s="17" t="str">
-        <x:v>Finance reflected order payment in cash/receivable totals.</x:v>
+      <x:c r="M12" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Finance shows ORD-000006 collection300 and balance1700. Total1750 includes prior fixtures.</x:t>
+        </x:is>
       </x:c>
       <x:c r="N12" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Finance GST page showed Cash in 200 for MTD and ORD-000011 receivable/payment summary.
+          <x:t xml:space="preserve">CH-6 2026-10-24 LOCAL: Finance shows ORD-000006 collection300 and balance1700. Total1750 includes prior fixtures. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
+Prior actual result: Finance reflected order payment in cash/receivable totals.
+Finance GST page showed Cash in 200 for MTD and ORD-000011 receivable/payment summary.
 CH-2 2026-10-21: Owner scenario: Finance showed order collection 300 and receivable 1700. Independent Finance-role session not tested. See docs_chat/CH2_BOUTIQUE_QA.md BA-011. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Finance shows ORD-000003 collection300/balance1700; aggregate cash850 includes earlier fixtures. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
 CH-4 2026-10-22 owner scenario: Finance shows ORD-000004 collection300 and balance1700. Aggregate1150 includes earlier local receipts. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
@@ -3993,12 +4037,16 @@
       <x:c r="L13" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="M13" s="17" t="str">
-        <x:v>GST report loaded and included GST-bearing QA order.</x:v>
+      <x:c r="M13" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">GST report loads; Include non-GST contains ORD-000006 with zeroGST. No GST-bearing calculation/export/filing acceptance.</x:t>
+        </x:is>
       </x:c>
       <x:c r="N13" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Finance GST page showed Output GST 180 and ORD-000011 in output GST list; XLSX export link present.
+          <x:t xml:space="preserve">CH-6 2026-10-24 LOCAL: GST report loads; Include non-GST contains ORD-000006 with zeroGST. No GST-bearing calculation/export/filing acceptance. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
+Prior actual result: GST report loaded and included GST-bearing QA order.
+Finance GST page showed Output GST 180 and ORD-000011 in output GST list; XLSX export link present.
 CH-2 2026-10-21: Owner scenario: GST report loaded and included non-GST order when selected. Zero-GST local fixture only: GST-bearing calculation, export and filing NOT tested. See docs_chat/CH2_BOUTIQUE_QA.md BA-012. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: GST report loads and includes non-GST ORD-000003. No GST-bearing calculation/export/filing claim. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
 CH-4 2026-10-22 owner scenario: GST report loads with the non-GST test order. No GST-bearing calculation, export or filing acceptance. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
@@ -4043,12 +4091,16 @@
       <x:c r="L14" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="M14" s="17" t="str">
-        <x:v>Queued sandbox WhatsApp tracking-link message and audit log.</x:v>
+      <x:c r="M14" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Native UI queued tracking email as dry-run only to ch6-qa@example.invalid. Flag and audit persisted. No external delivery.</x:t>
+        </x:is>
       </x:c>
       <x:c r="N14" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">communication_message_queue a2b4882e-e3b6-4616-bc2b-a57acc4ae030; log 8ebc4c2f-d2f2-48a5-8454-3620b8d43cdd; no live send.
+          <x:t xml:space="preserve">CH-6 2026-10-24 LOCAL: Native UI queued tracking email as dry-run only to ch6-qa@example.invalid. Flag and audit persisted. No external delivery. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
+Prior actual result: Queued sandbox WhatsApp tracking-link message and audit log.
+communication_message_queue a2b4882e-e3b6-4616-bc2b-a57acc4ae030; log 8ebc4c2f-d2f2-48a5-8454-3620b8d43cdd; no live send.
 CH-2 2026-10-21: Owner scenario: UI queued email tracking dry-run to ch2-qa@example.invalid; database dryRun=true and audit verified. No message delivered. See docs_chat/CH2_BOUTIQUE_QA.md BA-013. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Tracking email queued dry-run to ch3-qa@example.invalid; persisted dryRun/audit. No delivery. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
 CH-4 2026-10-22 owner scenario: Tracking email queued only as dry-run to ch4-qa@example.invalid. Dry-run flag and audit persisted. No delivery. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.
@@ -4093,12 +4145,16 @@
       <x:c r="L15" s="17" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="M15" s="17" t="str">
-        <x:v>Opened order detail/edit shell and saved harmless order notes edit.</x:v>
+      <x:c r="M15" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Native edit saved note ending edit verified. Total, receipt, measurement and workflow history preserved.</x:t>
+        </x:is>
       </x:c>
       <x:c r="N15" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">ORD-000012 notes updated to include "Edit smoke passed" without recalculating finance/production history.
+          <x:t xml:space="preserve">CH-6 2026-10-24 LOCAL: Native edit saved note ending edit verified. Total, receipt, measurement and workflow history preserved. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
+Prior actual result: Opened order detail/edit shell and saved harmless order notes edit.
+ORD-000012 notes updated to include "Edit smoke passed" without recalculating finance/production history.
 CH-2 2026-10-21: Owner scenario: edited order notes and reopened detail, total/payment/workflow preserved. See docs_chat/CH2_BOUTIQUE_QA.md BA-014. Historical V2-0 status/persona preconditions are not recertified.
 CH-3 2026-10-21 owner scenario: Edited notes; total/payment/fit/workflows preserved. See docs_chat/CH3_BOUTIQUE_QA.md. Independent role/GST preconditions not recertified.
 CH-4 2026-10-22 owner scenario: Edited notes. Payment, totals, measurements and workflow history preserved. See docs_chat/CH4_BOUTIQUE_QA.md. Historical persona/preconditions unchanged.

</xml_diff>

<commit_message>
Chat CH-7: add guarded notifications and daily summaries
</commit_message>
<xml_diff>
--- a/docs_v2/OS_PLUS_V2_QA_Test_Matrix.xlsx
+++ b/docs_v2/OS_PLUS_V2_QA_Test_Matrix.xlsx
@@ -3450,7 +3450,8 @@
       </x:c>
       <x:c r="N2" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">CH-6 2026-10-24 LOCAL: Retained owner-a Clerk session. A to B to A selection. B copied A order/customer/lead URLs return404. No fresh credential entry. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
+          <x:t xml:space="preserve">CH-7 2026-10-27 LOCAL Tier B: retained owner-a Clerk session; A to B to A and stale-tab refusal verified. Effective-role checks only; no fresh credential entry. See docs_chat/CH7_BOUTIQUE_QA.md.
+CH-6 2026-10-24 LOCAL: Retained owner-a Clerk session. A to B to A selection. B copied A order/customer/lead URLs return404. No fresh credential entry. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
 Prior actual result: Authenticated Owner/Admin opened Phantom Threads dashboard.
 Browser: localhost:3000/dashboard; Tenant Phantom Threads; role Owner/Admin.
 CH-2 2026-10-21: Owner-a existing authenticated session and tenant selector -&gt; Local QA A verified; fresh Clerk credential entry not repeated. See docs_chat/CH2_BOUTIQUE_QA.md BA-001. Historical V2-0 status/persona preconditions are not recertified.
@@ -3882,7 +3883,8 @@
       </x:c>
       <x:c r="N10" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">CH-6 2026-10-24 LOCAL: Browser public tracking plus separate anonymous HTTP200 exclude internal stages, worker, notes, receipt reference and email. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
+          <x:t xml:space="preserve">CH-7 2026-10-27 LOCAL Tier B: public tracking rendered two retained items; separate anonymous HTTP200 excluded internal stages, worker, notes, receipt reference and email. See docs_chat/CH7_BOUTIQUE_QA.md.
+CH-6 2026-10-24 LOCAL: Browser public tracking plus separate anonymous HTTP200 exclude internal stages, worker, notes, receipt reference and email. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
 Prior actual result: Opened public tracking link and verified customer-safe status.
 Tracking /track/TILaKurOoqN2o_dzXhSKK-cbmZkTos5D showed ORD-000011 and item status without internal worker data.
 CH-2 2026-10-21: Public tracking page rendered safe order/item status without internal worker, stage, payment or notes. Browser retained login; no fresh anonymous browser claim. See docs_chat/CH2_BOUTIQUE_QA.md BA-009. Historical V2-0 status/persona preconditions are not recertified.
@@ -4152,7 +4154,8 @@
       </x:c>
       <x:c r="N15" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">CH-6 2026-10-24 LOCAL: Native edit saved note ending edit verified. Total, receipt, measurement and workflow history preserved. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
+          <x:t xml:space="preserve">CH-7 2026-10-27 LOCAL Tier B: opened ORD-000006 detail/edit without saving; production page loaded. Read-only SQL preserved total2000, one prior receipt300, balance1700, two workflows and stage history. Not a new 14-check run. See docs_chat/CH7_BOUTIQUE_QA.md.
+CH-6 2026-10-24 LOCAL: Native edit saved note ending edit verified. Total, receipt, measurement and workflow history preserved. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
 Prior actual result: Opened order detail/edit shell and saved harmless order notes edit.
 ORD-000012 notes updated to include "Edit smoke passed" without recalculating finance/production history.
 CH-2 2026-10-21: Owner scenario: edited order notes and reopened detail, total/payment/workflow preserved. See docs_chat/CH2_BOUTIQUE_QA.md BA-014. Historical V2-0 status/persona preconditions are not recertified.

</xml_diff>

<commit_message>
Chat CH-8: add guarded local voice-note processing
</commit_message>
<xml_diff>
--- a/docs_v2/OS_PLUS_V2_QA_Test_Matrix.xlsx
+++ b/docs_v2/OS_PLUS_V2_QA_Test_Matrix.xlsx
@@ -3450,7 +3450,8 @@
       </x:c>
       <x:c r="N2" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">CH-7 2026-10-27 LOCAL Tier B: retained owner-a Clerk session; A to B to A and stale-tab refusal verified. Effective-role checks only; no fresh credential entry. See docs_chat/CH7_BOUTIQUE_QA.md.
+          <x:t xml:space="preserve">CH-8 2026-10-27 LOCAL Tier B: retained owner-a Clerk session; Authenticated owner and effective-role checks; two-tenant voice QA passed. Effective-role checks only; no fresh credential entry. See docs_chat/CH8_BOUTIQUE_QA.md.
+CH-7 2026-10-27 LOCAL Tier B: retained owner-a Clerk session; A to B to A and stale-tab refusal verified. Effective-role checks only; no fresh credential entry. See docs_chat/CH7_BOUTIQUE_QA.md.
 CH-6 2026-10-24 LOCAL: Retained owner-a Clerk session. A to B to A selection. B copied A order/customer/lead URLs return404. No fresh credential entry. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
 Prior actual result: Authenticated Owner/Admin opened Phantom Threads dashboard.
 Browser: localhost:3000/dashboard; Tenant Phantom Threads; role Owner/Admin.
@@ -3883,7 +3884,8 @@
       </x:c>
       <x:c r="N10" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">CH-7 2026-10-27 LOCAL Tier B: public tracking rendered two retained items; separate anonymous HTTP200 excluded internal stages, worker, notes, receipt reference and email. See docs_chat/CH7_BOUTIQUE_QA.md.
+          <x:t xml:space="preserve">CH-8 2026-10-27 LOCAL Tier B: public tracking rendered two retained items; separate anonymous HTTP200 excluded internal stages, worker, notes, receipt reference and email. See docs_chat/CH8_BOUTIQUE_QA.md.
+CH-7 2026-10-27 LOCAL Tier B: public tracking rendered two retained items; separate anonymous HTTP200 excluded internal stages, worker, notes, receipt reference and email. See docs_chat/CH7_BOUTIQUE_QA.md.
 CH-6 2026-10-24 LOCAL: Browser public tracking plus separate anonymous HTTP200 exclude internal stages, worker, notes, receipt reference and email. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
 Prior actual result: Opened public tracking link and verified customer-safe status.
 Tracking /track/TILaKurOoqN2o_dzXhSKK-cbmZkTos5D showed ORD-000011 and item status without internal worker data.
@@ -4154,7 +4156,8 @@
       </x:c>
       <x:c r="N15" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">CH-7 2026-10-27 LOCAL Tier B: opened ORD-000006 detail/edit without saving; production page loaded. Read-only SQL preserved total2000, one prior receipt300, balance1700, two workflows and stage history. Not a new 14-check run. See docs_chat/CH7_BOUTIQUE_QA.md.
+          <x:t xml:space="preserve">CH-8 2026-10-27 LOCAL Tier B: opened ORD-000006 detail/edit without saving; production page loaded. Read-only SQL preserved total2000, one prior receipt300, balance1700, two workflows and stage history. Not a new 14-check run. See docs_chat/CH8_BOUTIQUE_QA.md.
+CH-7 2026-10-27 LOCAL Tier B: opened ORD-000006 detail/edit without saving; production page loaded. Read-only SQL preserved total2000, one prior receipt300, balance1700, two workflows and stage history. Not a new 14-check run. See docs_chat/CH7_BOUTIQUE_QA.md.
 CH-6 2026-10-24 LOCAL: Native edit saved note ending edit verified. Total, receipt, measurement and workflow history preserved. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
 Prior actual result: Opened order detail/edit shell and saved harmless order notes edit.
 ORD-000012 notes updated to include "Edit smoke passed" without recalculating finance/production history.

</xml_diff>

<commit_message>
Chat CH-9: add safe website capture and focused settings
</commit_message>
<xml_diff>
--- a/docs_v2/OS_PLUS_V2_QA_Test_Matrix.xlsx
+++ b/docs_v2/OS_PLUS_V2_QA_Test_Matrix.xlsx
@@ -3450,7 +3450,8 @@
       </x:c>
       <x:c r="N2" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">CH-8 2026-10-27 LOCAL Tier B: retained owner-a Clerk session; Authenticated owner and effective-role checks; two-tenant voice QA passed. Effective-role checks only; no fresh credential entry. See docs_chat/CH8_BOUTIQUE_QA.md.
+          <x:t xml:space="preserve">CH-9 2026-10-28 LOCAL Tier B: retained owner-a Clerk session and normal A to B to A selector. Effective manager/viewer/finance checks passed; original membership and grants restored. No fresh credential login. See docs_chat/CH9_BOUTIQUE_QA.md.
+CH-8 2026-10-27 LOCAL Tier B: retained owner-a Clerk session; Authenticated owner and effective-role checks; two-tenant voice QA passed. Effective-role checks only; no fresh credential entry. See docs_chat/CH8_BOUTIQUE_QA.md.
 CH-7 2026-10-27 LOCAL Tier B: retained owner-a Clerk session; A to B to A and stale-tab refusal verified. Effective-role checks only; no fresh credential entry. See docs_chat/CH7_BOUTIQUE_QA.md.
 CH-6 2026-10-24 LOCAL: Retained owner-a Clerk session. A to B to A selection. B copied A order/customer/lead URLs return404. No fresh credential entry. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
 Prior actual result: Authenticated Owner/Admin opened Phantom Threads dashboard.
@@ -3884,7 +3885,8 @@
       </x:c>
       <x:c r="N10" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">CH-8 2026-10-27 LOCAL Tier B: public tracking rendered two retained items; separate anonymous HTTP200 excluded internal stages, worker, notes, receipt reference and email. See docs_chat/CH8_BOUTIQUE_QA.md.
+          <x:t xml:space="preserve">CH-9 2026-10-28 LOCAL Tier B: two-item public tracking rendered. Anonymous HTTP200 excludes internal stages, worker, notes, receipt reference and email. See docs_chat/CH9_BOUTIQUE_QA.md.
+CH-8 2026-10-27 LOCAL Tier B: public tracking rendered two retained items; separate anonymous HTTP200 excluded internal stages, worker, notes, receipt reference and email. See docs_chat/CH8_BOUTIQUE_QA.md.
 CH-7 2026-10-27 LOCAL Tier B: public tracking rendered two retained items; separate anonymous HTTP200 excluded internal stages, worker, notes, receipt reference and email. See docs_chat/CH7_BOUTIQUE_QA.md.
 CH-6 2026-10-24 LOCAL: Browser public tracking plus separate anonymous HTTP200 exclude internal stages, worker, notes, receipt reference and email. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
 Prior actual result: Opened public tracking link and verified customer-safe status.
@@ -4156,7 +4158,8 @@
       </x:c>
       <x:c r="N15" s="17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">CH-8 2026-10-27 LOCAL Tier B: opened ORD-000006 detail/edit without saving; production page loaded. Read-only SQL preserved total2000, one prior receipt300, balance1700, two workflows and stage history. Not a new 14-check run. See docs_chat/CH8_BOUTIQUE_QA.md.
+          <x:t xml:space="preserve">CH-9 2026-10-28 LOCAL Tier B: ORD-000006 detail/editor opened without saving; production loaded. Read-only checks preserve total2000, paid300, balance1700, two workflows, fit reference and stage history. Not a new full14-check run. See docs_chat/CH9_BOUTIQUE_QA.md.
+CH-8 2026-10-27 LOCAL Tier B: opened ORD-000006 detail/edit without saving; production page loaded. Read-only SQL preserved total2000, one prior receipt300, balance1700, two workflows and stage history. Not a new 14-check run. See docs_chat/CH8_BOUTIQUE_QA.md.
 CH-7 2026-10-27 LOCAL Tier B: opened ORD-000006 detail/edit without saving; production page loaded. Read-only SQL preserved total2000, one prior receipt300, balance1700, two workflows and stage history. Not a new 14-check run. See docs_chat/CH7_BOUTIQUE_QA.md.
 CH-6 2026-10-24 LOCAL: Native edit saved note ending edit verified. Total, receipt, measurement and workflow history preserved. See docs_chat/CH6_BOUTIQUE_QA.md. Effective-role QA is not independent role sign-in.
 Prior actual result: Opened order detail/edit shell and saved harmless order notes edit.

</xml_diff>